<commit_message>
Actualización electrónica (Modulo Power mb v2)
</commit_message>
<xml_diff>
--- a/Test_profile.xlsx
+++ b/Test_profile.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f3f9d6c30eef4a4/Documentos/UPM/4º/TFG/GitFlexBench/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_7251E617CF19DFBF2E0BB744F2012D16110D1170" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB4DC350-C6AD-493E-BD70-81BD88599D7C}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_7251E617CF19DFBF2E0BB744F2012D16110D1170" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E7F6995-DB74-4853-A90C-9836DADE6453}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="27" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="18" uniqueCount="7">
   <si>
     <t>Nombre_Perfil</t>
   </si>
@@ -34,22 +34,13 @@
     <t>Max</t>
   </si>
   <si>
-    <t>Standard L</t>
-  </si>
-  <si>
-    <t>Standard M</t>
-  </si>
-  <si>
-    <t>Standard S</t>
+    <t>Normal Test</t>
+  </si>
+  <si>
+    <t>Try</t>
   </si>
   <si>
     <t>Test</t>
-  </si>
-  <si>
-    <t>Prueba Rapida</t>
-  </si>
-  <si>
-    <t>Prueba</t>
   </si>
 </sst>
 </file>
@@ -67,12 +58,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.24997711111789"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -88,9 +85,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
@@ -107,10 +112,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -430,112 +431,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="true"/>
-    <col min="2" max="2" width="4.109375" customWidth="true"/>
-    <col min="3" max="3" width="4.5546875" customWidth="true"/>
-    <col min="4" max="4" width="5.77734375" customWidth="true"/>
+    <col min="1" max="1" width="12.88671875" style="1" customWidth="true"/>
+    <col min="2" max="2" width="5" style="1" customWidth="true"/>
+    <col min="3" max="3" width="5" style="1" customWidth="true"/>
+    <col min="4" max="4" width="5.77734375" style="1" customWidth="true"/>
   </cols>
   <sheetData>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="0">
-        <v>180</v>
-      </c>
-      <c r="C2" s="0">
-        <v>300</v>
-      </c>
-      <c r="D2" s="0">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1">
+        <v>5700</v>
+      </c>
+      <c r="C2" s="1">
+        <v>9700</v>
+      </c>
+      <c r="D2" s="1">
         <v>20</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="0">
-        <v>180</v>
-      </c>
-      <c r="C3" s="0">
-        <v>300</v>
-      </c>
-      <c r="D3" s="0">
-        <v>30</v>
+      <c r="B3" s="1">
+        <v>0</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2000</v>
+      </c>
+      <c r="D3" s="1">
+        <v>20</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="0">
-        <v>180</v>
-      </c>
-      <c r="C4" s="0">
-        <v>300</v>
-      </c>
-      <c r="D4" s="0">
-        <v>40</v>
+      <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1200</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2400</v>
+      </c>
+      <c r="D4" s="1">
+        <v>20</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="0">
-        <v>180</v>
-      </c>
-      <c r="C5" s="0">
-        <v>300</v>
-      </c>
-      <c r="D5" s="0">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="0">
-        <v>0</v>
-      </c>
-      <c r="C6" s="0">
-        <v>50</v>
-      </c>
-      <c r="D6" s="0">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="0">
-        <v>0</v>
-      </c>
-      <c r="C7" s="0">
-        <v>50</v>
-      </c>
-      <c r="D7" s="0">
-        <v>2</v>
-      </c>
+      <c r="A5" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>